<commit_message>
Manual RECEIVE: AI NUC (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaction Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Batches" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transaction Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +476,26 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Serial Number</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Reference No.</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Source Document</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Delivery Address</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -584,6 +604,51 @@
           <t>Active</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Top floor</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>160</v>
+      </c>
+      <c r="G5" t="n">
+        <v>160</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -596,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -660,6 +725,31 @@
           <t>Storage Location</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Serial Number</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Reference No.</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Document Type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Delivery Address</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Source Document</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1038,6 +1128,70 @@
           <t>[{"batch_id": 2, "date_received": "2026-07-31", "qty_taken": 30}]</t>
         </is>
       </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-06T05:11:13.426512+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Manual form entry: RECEIVE 160.0 units AI NUC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>160</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 4}]</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Top floor</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Log rejected message (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -645,10 +645,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -661,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1178,20 +1174,55 @@
           <t>[{"batch_id": 4}]</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>MANUAL_FORM</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>Top floor</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-06T05:51:52.468065+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>all products dispatched</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Manual DISPATCH: AI NUC (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -630,14 +630,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>160</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1201,7 +1201,6 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>krish</t>
@@ -1217,12 +1216,66 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-06T05:52:21.127501+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Manual form entry: DISPATCH 160.0 units AI NUC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>160</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 4, "date_received": "Top floor", "qty_taken": 160}]</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Manual TRANSFER: AI NUC (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,18 +633,59 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Depleted</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Depleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ghatkopar</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Top floor</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>10</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Depleted</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -657,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1353,16 +1394,76 @@
           <t>[{"batch_id": 4, "date_received": "Top floor", "qty_taken": 150.0}]</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>MANUAL_FORM</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-06T06:03:14.630555+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Manual form entry: TRANSFER 10.0 units AI NUC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TRANSFER</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ghatkopar</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>{"consumed": [{"batch_id": 4, "date_received": "Top floor", "qty_taken": 10}], "created_batch_ids": [5]}</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Manual ADJUST: AI NUC (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,10 +722,47 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>500</v>
+      </c>
+      <c r="G8" t="n">
+        <v>500</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -738,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1549,20 +1586,76 @@
           <t>[{"batch_id": 6}]</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>MANUAL_FORM</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>g floor</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-06T06:06:30.786989+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Manual form entry: ADJUST 500.0 units AI NUC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ADJUST</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>500</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 7}]</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Manual RECEIVE: SSD (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -547,9 +547,55 @@
           <t>ABC123</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Top floor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>500</v>
+      </c>
+      <c r="G3" t="n">
+        <v>500</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>ABC124</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -562,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1378,19 +1424,84 @@
           <t>ABC123</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>MANUAL_FORM</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>Store room</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:12:14.598091+00:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Manual form entry: RECEIVE 500.0 units SSD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>500</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 2}]</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>ABC124</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Top floor</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
RECEIVE: recieved 200 ram sticks in bhiwandi kept in store room (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -593,6 +593,51 @@
           <t>ABC124</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ram sticks</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>store room</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>200</v>
+      </c>
+      <c r="G4" t="n">
+        <v>200</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -605,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1513,7 +1558,6 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>krish</t>
@@ -1529,12 +1573,66 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:13:07.756902+00:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>recieved 200 ram sticks in bhiwandi kept in store room</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ram sticks</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>200</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 3}]</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>store room</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
TRANSFER: transfered 100 ai nuc from bhiwandi to ghatkopar store room (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -527,14 +527,14 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>100</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -634,10 +634,47 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ghatkopar</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Store room</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -650,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1623,16 +1660,72 @@
           <t>[{"batch_id": 3}]</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>store room</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:13:41.408087+00:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>transfered 100 ai nuc from bhiwandi to ghatkopar store room</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TRANSFER</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Ghatkopar</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>100</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>{"consumed": [{"batch_id": 1, "date_received": "Store room", "qty_taken": 100}], "created_batch_ids": [4]}</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DISPATCH: sold ai nuc 100 pieces from ghatkopar (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -649,21 +649,20 @@
           <t>Ghatkopar</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Store room</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>100</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -671,10 +670,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -687,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1720,12 +1715,62 @@
           <t>{"consumed": [{"batch_id": 1, "date_received": "Store room", "qty_taken": 100}], "created_batch_ids": [4]}</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:15:46.281615+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>sold ai nuc 100 pieces from ghatkopar</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>AI NUC</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ghatkopar</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>pieces</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 4, "date_received": "None", "qty_taken": 100}]</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Manual DISPATCH: SSD (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -576,7 +576,7 @@
         <v>500</v>
       </c>
       <c r="G3" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1815,16 +1815,71 @@
           <t>[{"batch_id": 1, "date_received": "Store room", "qty_taken": 100.0}]</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>MANUAL_FORM</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:25:35.411049+00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Manual form entry: DISPATCH 250.0 units SSD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>250</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 2, "date_received": "Top floor", "qty_taken": 250.0}]</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DISPATCH: dispatch ssd from bhiwandi 150 quantity (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -576,7 +576,7 @@
         <v>500</v>
       </c>
       <c r="G3" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1870,16 +1870,67 @@
           <t>[{"batch_id": 2, "date_received": "Top floor", "qty_taken": 250.0}]</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>MANUAL_FORM</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:26:57.667044+00:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>dispatch ssd from bhiwandi 150 quantity</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ssd</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>150</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 2, "date_received": "Top floor", "qty_taken": 150}]</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Manual RECEIVE: Ram sticks (krish)
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -670,6 +670,51 @@
           <t>Active</t>
         </is>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ram sticks</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>g floor</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -682,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1925,12 +1970,70 @@
           <t>[{"batch_id": 2, "date_received": "Top floor", "qty_taken": 150}]</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-06T11:42:14.729672+00:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Manual form entry: RECEIVE 1.0 units Ram sticks</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RECEIVE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ram sticks</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>[{"batch_id": 5}]</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>MANUAL_FORM</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>g floor</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Receive: Krish [TXN-000001] by Panache Digilife Limited
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inwards" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inward Lines" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serials" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work Orders" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaction Log" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Meta" sheetId="10" state="hidden" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Journal" sheetId="11" state="hidden" r:id="rId11"/>
+    <sheet name="Items" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inwards" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Inward Lines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Batches" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Serials" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Work Orders" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Consumption" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Transaction Log" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="_Meta" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet name="_Journal" sheetId="11" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -533,6 +533,54 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:17:03+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -544,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -573,6 +621,66 @@
         <is>
           <t>2</t>
         </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>txn</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>grn2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -586,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -634,6 +742,141 @@
           <t>Old Value</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B0000001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>L0000001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Inward Lines</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001-01</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Inwards</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -718,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -923,6 +1166,80 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2005-10-22</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Ashwin</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PDLKDLAVK123</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Panache Digilife Limited</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:17:03+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -934,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1085,6 +1402,84 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>QC_HOLD</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Rack 05</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>B0000001</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1096,7 +1491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1238,6 +1633,99 @@
       <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Created At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B0000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>QC_HOLD</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Rack 05</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2005-10-22</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:17:03+05:30</t>
         </is>
       </c>
     </row>
@@ -1618,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1751,6 +2239,91 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>L0000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:17:03+05:30</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>QC_HOLD</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Rack 05</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Ashwin</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>PDLKDLAVK123</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Panache Digilife Limited</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>CBU inward</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
QC B0000001 [TXN-000002] by krish
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -767,8 +767,6 @@
           <t>ITM-00001</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -794,8 +792,6 @@
           <t>B0000001</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -821,8 +817,6 @@
           <t>L0000001</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -848,8 +842,6 @@
           <t>GRN-2026-0001-01</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -875,8 +867,165 @@
           <t>GRN-2026-0001</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B0000001</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 5, "Status": "Active"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>B0000002</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L0000002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Inward Lines</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001-01</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>{"QC Status": "PENDING"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Inwards</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{"QC Status": "PENDING"}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1204,7 +1353,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="X2" t="n">
@@ -1468,7 +1617,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -1491,7 +1640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1681,51 +1830,149 @@
         <v>5</v>
       </c>
       <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Depleted</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TXN-000001</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:17:03+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B0000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Rack 05</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2005-10-22</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
         <v>5</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>units</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>GRN-2026-0001</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>CBU</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>INWARD</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>TXN-000001</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>2026-10-09T16:17:03+05:30</t>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>QC_PASS</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>B0000001</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:45:16+05:30</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2324,6 +2571,86 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>L0000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TXN-000002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:45:16+05:30</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>QC_PASS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>GRN-2026-0001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>QC_HOLD</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Rack 05</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Chat dispatch: 5 krish sold from mbhiwandi to abc [TXN-000003] by krish
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -927,8 +927,6 @@
           <t>B0000002</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -954,8 +952,6 @@
           <t>L0000002</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1026,6 +1022,68 @@
           <t>{"QC Status": "PENDING"}</t>
         </is>
       </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TXN-000003</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>B0000002</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 5, "Status": "Active"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TXN-000003</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L0000003</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1923,7 +1981,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -1932,7 +1990,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2353,7 +2411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2651,6 +2709,76 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>L0000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TXN-000003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-10-09T16:45:30+05:30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ITM-00001</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Krish</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Sale / customer dispatch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Receive: abc [TXN-000004] by krish
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -581,6 +581,54 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ITM-00002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:02:11+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -630,7 +678,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -640,7 +688,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -650,7 +698,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -660,7 +708,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -670,7 +718,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -680,7 +728,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -694,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1082,8 +1130,141 @@
           <t>L0000003</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ITM-00002</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>B0000003</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L0000004</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Inward Lines</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002-01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Inwards</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1168,7 +1349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG2"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1447,6 +1628,75 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:02:11+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1458,7 +1708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1687,6 +1937,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ITM-00002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>50</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>B0000003</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1698,7 +2026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2031,6 +2359,99 @@
       <c r="W3" t="inlineStr">
         <is>
           <t>2026-10-09T16:45:16+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B0000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ITM-00002</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:02:11+05:30</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2779,6 +3200,86 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>L0000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TXN-000004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:02:11+05:30</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GRN-2026-0002</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ITM-00002</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>CBU inward</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dispatch: abc [TXN-000005] by krish
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -718,7 +718,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -742,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1155,8 +1155,6 @@
           <t>ITM-00002</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1182,8 +1180,6 @@
           <t>B0000003</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1209,8 +1205,6 @@
           <t>L0000004</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1236,8 +1230,6 @@
           <t>GRN-2026-0002-01</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1263,8 +1255,68 @@
           <t>GRN-2026-0002</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TXN-000005</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>B0000003</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 50, "Status": "Active"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TXN-000005</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L0000005</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2407,7 +2459,7 @@
         <v>50</v>
       </c>
       <c r="J4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -2416,7 +2468,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -2832,7 +2884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3280,6 +3332,76 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>L0000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TXN-000005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:02:27+05:30</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ITM-00002</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>50</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Sale / customer dispatch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Receive: PCIe Card 1ch [TXN-000006] by Rajesh
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -629,6 +629,54 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pcie card 1ch</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-10-21T16:07:29+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -678,7 +726,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -688,7 +736,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -698,7 +746,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -708,7 +756,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -718,7 +766,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -728,7 +776,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -742,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1315,8 +1363,141 @@
           <t>L0000005</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>B0000004</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L0000006</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Inward Lines</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003-01</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Inwards</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1401,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG3"/>
+  <dimension ref="A1:AG4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1749,6 +1930,80 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Yuan High tech Development Co. Ltd</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>YN2610011</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>2026-10-21T16:07:29+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1760,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2067,6 +2322,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>pallet</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>B0000004</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2078,7 +2411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2504,6 +2837,99 @@
       <c r="W4" t="inlineStr">
         <is>
           <t>2026-10-16T12:02:11+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B0000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>pallet</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>7</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2026-10-21T16:07:29+05:30</t>
         </is>
       </c>
     </row>
@@ -2884,7 +3310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3402,6 +3828,91 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L0000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TXN-000006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-10-21T16:07:29+05:30</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GRN-2026-0003</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>pallet</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yuan High tech Development Co. Ltd</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>YN2610011</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>CBU inward</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Receive: ASUS Laptop [TXN-000007] by Rajesh
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -677,6 +677,54 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ASUS Laptop</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>asus laptop</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:54:23+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -726,7 +774,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -736,7 +784,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -746,7 +794,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -756,7 +804,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -766,7 +814,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -776,7 +824,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -790,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1388,8 +1436,6 @@
           <t>ITM-00003</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1415,8 +1461,6 @@
           <t>B0000004</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1442,8 +1486,6 @@
           <t>L0000006</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1469,8 +1511,6 @@
           <t>GRN-2026-0003-01</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1496,8 +1536,141 @@
           <t>GRN-2026-0003</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>B0000005</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L0000007</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Inward Lines</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004-01</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Inwards</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1582,7 +1755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AG5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2004,6 +2177,85 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Asus india Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ASINBH0206</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>260520562023</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>152</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:54:23+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2015,7 +2267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2400,6 +2652,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ASUS Laptop</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>152</v>
+      </c>
+      <c r="H5" t="n">
+        <v>152</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>152</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>B0000005</t>
+        </is>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2411,7 +2741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2930,6 +3260,99 @@
       <c r="W5" t="inlineStr">
         <is>
           <t>2026-10-21T16:07:29+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B0000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ASUS Laptop</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>152</v>
+      </c>
+      <c r="J6" t="n">
+        <v>152</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:54:23+05:30</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3913,6 +4336,91 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L0000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TXN-000007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:54:23+05:30</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GRN-2026-0004</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ASUS Laptop</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>152</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Asus india Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>ASINBH0206</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>CBU inward</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dispatch: ASUS Laptop [TXN-000008] by Rajesh
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1561,8 +1561,6 @@
           <t>ITM-00004</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1588,8 +1586,6 @@
           <t>B0000005</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1615,8 +1611,6 @@
           <t>L0000007</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1642,8 +1636,6 @@
           <t>GRN-2026-0004-01</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1669,8 +1661,68 @@
           <t>GRN-2026-0004</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TXN-000008</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>B0000005</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 152}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TXN-000008</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L0000008</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3308,7 +3360,7 @@
         <v>152</v>
       </c>
       <c r="J6" t="n">
-        <v>152</v>
+        <v>4</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3733,7 +3785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4421,6 +4473,91 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L0000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TXN-000008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:55:35+05:30</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PDL/BH/10/27/092</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ASUS Laptop</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>148</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Asus India Pvt ltd</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>PDL/BH/10/27/092</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Sale / customer dispatch</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Padgha</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dispatch: ASUS Laptop [TXN-000009] by Rajesh
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1721,8 +1721,68 @@
           <t>L0000008</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TXN-000009</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>B0000005</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 4, "Status": "Active"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TXN-000009</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L0000009</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3360,7 +3420,7 @@
         <v>152</v>
       </c>
       <c r="J6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3369,7 +3429,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -3785,7 +3845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4558,6 +4618,76 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>L0000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TXN-000009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:56:05+05:30</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ITM-00004</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ASUS Laptop</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Asus India Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Sale / customer dispatch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Dispatch: PCIe Card 1ch [TXN-000010] by Rajesh
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1781,8 +1781,68 @@
           <t>L0000009</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>TXN-000010</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>B0000004</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 7, "Status": "Active"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>TXN-000010</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L0000010</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3327,7 +3387,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -3336,7 +3396,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -3845,7 +3905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4688,6 +4748,91 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>L0000010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TXN-000010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-10-21T18:58:37+05:30</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PDL/MH/10/27/045</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Esbee Dynamed Pvt ltd</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>PDL/MH/10/27/045</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Sale / customer dispatch</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Govandi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Receive: PCIe Card 1ch [TXN-000011] by krish
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -66,11 +66,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -774,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -784,7 +785,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -804,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -814,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -824,7 +825,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -838,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1841,8 +1842,114 @@
           <t>L0000010</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>B0000006</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L0000011</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Inward Lines</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005-01</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Inwards</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1927,7 +2034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG5"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2131,6 +2238,16 @@
           <t>Created At</t>
         </is>
       </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>Transporter Name</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>Docket No</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2425,6 +2542,75 @@
       <c r="AG5" t="inlineStr">
         <is>
           <t>2026-10-21T18:54:23+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>2026-10-23T11:24:08+05:30</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:X6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2902,6 +3088,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>B0000006</t>
+        </is>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2913,7 +3177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3528,6 +3792,99 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B0000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>CBU</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>2026-10-23T11:24:08+05:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3539,7 +3896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3669,6 +4026,16 @@
       <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Updated At</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Transporter Name</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Docket No</t>
         </is>
       </c>
     </row>
@@ -3905,7 +4272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4037,6 +4404,26 @@
           <t>Remarks</t>
         </is>
       </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Transporter Name</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Docket No</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>Last Edited By</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>Last Edited At</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4830,6 +5217,86 @@
       <c r="U11" t="inlineStr">
         <is>
           <t>Govandi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L0000011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TXN-000011</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-10-23T11:24:08+05:30</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>GRN-2026-0005</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>CBU inward</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dispatch: PCIe Card 1ch [TXN-000012] by krish
</commit_message>
<xml_diff>
--- a/data/inventory_data.xlsx
+++ b/data/inventory_data.xlsx
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1867,8 +1867,6 @@
           <t>B0000006</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1894,8 +1892,6 @@
           <t>L0000011</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1921,8 +1917,6 @@
           <t>GRN-2026-0005-01</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1948,8 +1942,68 @@
           <t>GRN-2026-0005</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TXN-000012</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>B0000006</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>{"Qty Remaining": 2, "Status": "Active"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TXN-000012</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>append</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Transaction Log</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L0000012</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3837,7 +3891,7 @@
         <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3846,7 +3900,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Depleted</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -4272,7 +4326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5300,6 +5354,76 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L0000012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TXN-000012</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-10-23T11:24:41+05:30</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>DISPATCH</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ITM-00003</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PCIe Card 1ch</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Bhiwandi</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FG_STORE</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>krish</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Sale / customer dispatch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>